<commit_message>
Update Policy 7 TIMESLICE from ANNUAL to DAYNIGHT
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_RES_SHARE_50%_24_7_LO.xlsx
+++ b/SuppXLS/Scen_RES_SHARE_50%_24_7_LO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yukiainge/Documents/Claude/Projects/Energy Modeling &amp; Climate Policy/05_TIMES_Modeling/models/Models MSc_SELECT_updated-20260612/SuppXLS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E18FC40-6F1D-3744-8ABC-B056AA4596BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CC0FEA-185C-5C4A-85AF-4E48CC5A0771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -91,10 +91,10 @@
     <t>FLO_SHAR</t>
   </si>
   <si>
-    <t>ANNUAL</t>
+    <t>LO</t>
   </si>
   <si>
-    <t>LO</t>
+    <t>DAYNITE</t>
   </si>
 </sst>
 </file>
@@ -4484,7 +4484,7 @@
     </row>
     <row r="6" spans="2:9">
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>9</v>
@@ -4499,7 +4499,7 @@
         <v>2030</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6" s="5">
         <v>0.5</v>

</xml_diff>

<commit_message>
add milestone yrs in 7 and remove onshore wind cap
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_RES_SHARE_50%_24_7_LO.xlsx
+++ b/SuppXLS/Scen_RES_SHARE_50%_24_7_LO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yukiainge/Documents/Claude/Projects/Energy Modeling &amp; Climate Policy/05_TIMES_Modeling/models/Models MSc_SELECT_updated-20260612/SuppXLS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85CC0FEA-185C-5C4A-85AF-4E48CC5A0771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3007C30A-F967-AB48-A8CC-1B4B453D979C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Year</t>
   </si>
@@ -95,6 +95,9 @@
   </si>
   <si>
     <t>DAYNITE</t>
+  </si>
+  <si>
+    <t>2023,2025, 2030, 2035, 2040, 2045, 2050</t>
   </si>
 </sst>
 </file>
@@ -4495,8 +4498,8 @@
       <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="2">
-        <v>2030</v>
+      <c r="F6" t="s">
+        <v>13</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>11</v>

</xml_diff>